<commit_message>
矫正 	modified:   notebook/help.ipynb 	modified:   "notebook/\345\260\217\351\254\274\350\220\275\347\202\271/\345\260\217\351\254\274\350\220\275\347\202\271.ipynb" 	modified:   "notebook/\345\260\217\351\254\274\350\220\275\347\202\271/\350\220\275\347\202\271\347\273\223\350\256\272.xlsx"
</commit_message>
<xml_diff>
--- a/notebook/小鬼落点/落点结论.xlsx
+++ b/notebook/小鬼落点/落点结论.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowHeight="17775"/>
+    <workbookView windowWidth="21225" windowHeight="12615"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="19">
   <si>
     <t>场地</t>
   </si>
@@ -98,7 +98,7 @@
     <numFmt numFmtId="176" formatCode="0.0000000000_ "/>
     <numFmt numFmtId="177" formatCode="0.0000_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,13 +109,6 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -583,152 +576,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -741,6 +734,9 @@
     <xf numFmtId="177" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1090,7 +1086,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="2" width="5.375" customWidth="1"/>
@@ -1221,28 +1217,28 @@
         <v>9</v>
       </c>
       <c r="B5" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="6">
+        <v>-10</v>
+      </c>
+      <c r="E5" s="6">
         <v>70</v>
       </c>
-      <c r="E5" s="6">
-        <v>150</v>
-      </c>
       <c r="F5" s="7">
-        <v>404</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G5" s="7">
-        <v>700.9999389648</v>
+        <v>407.9999694824</v>
       </c>
       <c r="H5" s="8">
-        <v>3.475</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>11</v>
+        <v>3.425</v>
+      </c>
+      <c r="I5" s="8">
+        <v>7.975</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1250,28 +1246,28 @@
         <v>9</v>
       </c>
       <c r="B6" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D6" s="6">
-        <v>70</v>
+        <v>-10</v>
       </c>
       <c r="E6" s="6">
-        <v>149</v>
+        <v>69</v>
       </c>
       <c r="F6" s="7">
-        <v>404</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G6" s="7">
-        <v>696.9999389648</v>
+        <v>406.9999694824</v>
       </c>
       <c r="H6" s="8">
-        <v>3.475</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>11</v>
+        <v>3.425</v>
+      </c>
+      <c r="I6" s="8">
+        <v>7.9625</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1282,22 +1278,22 @@
         <v>2</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D7" s="6">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7" s="6">
         <v>150</v>
       </c>
       <c r="F7" s="7">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G7" s="7">
         <v>700.9999389648</v>
       </c>
       <c r="H7" s="8">
-        <v>3.4875</v>
+        <v>3.475</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>11</v>
@@ -1311,22 +1307,22 @@
         <v>2</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" s="6">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E8" s="6">
         <v>149</v>
       </c>
       <c r="F8" s="7">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="G8" s="7">
         <v>696.9999389648</v>
       </c>
       <c r="H8" s="8">
-        <v>3.4875</v>
+        <v>3.475</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>11</v>
@@ -1337,25 +1333,25 @@
         <v>9</v>
       </c>
       <c r="B9" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D9" s="6">
+        <v>71</v>
+      </c>
+      <c r="E9" s="6">
         <v>150</v>
       </c>
-      <c r="E9" s="6">
-        <v>230</v>
-      </c>
       <c r="F9" s="7">
-        <v>500.0000305176</v>
+        <v>405</v>
       </c>
       <c r="G9" s="7">
-        <v>817.9999389648</v>
+        <v>700.9999389648</v>
       </c>
       <c r="H9" s="8">
-        <v>4.675</v>
+        <v>3.4875</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>11</v>
@@ -1366,25 +1362,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D10" s="6">
-        <v>150</v>
+        <v>71</v>
       </c>
       <c r="E10" s="6">
-        <v>229</v>
+        <v>149</v>
       </c>
       <c r="F10" s="7">
-        <v>500.0000305176</v>
+        <v>405</v>
       </c>
       <c r="G10" s="7">
-        <v>817.9999389648</v>
+        <v>696.9999389648</v>
       </c>
       <c r="H10" s="8">
-        <v>4.675</v>
+        <v>3.4875</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>11</v>
@@ -1398,10 +1394,10 @@
         <v>3</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="6">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E11" s="6">
         <v>230</v>
@@ -1427,10 +1423,10 @@
         <v>3</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D12" s="6">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E12" s="6">
         <v>229</v>
@@ -1453,25 +1449,25 @@
         <v>9</v>
       </c>
       <c r="B13" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D13" s="6">
+        <v>151</v>
+      </c>
+      <c r="E13" s="6">
         <v>230</v>
       </c>
-      <c r="E13" s="6">
-        <v>310</v>
-      </c>
       <c r="F13" s="7">
-        <v>681</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G13" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H13" s="8">
-        <v>6.9375</v>
+        <v>4.675</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>11</v>
@@ -1482,25 +1478,25 @@
         <v>9</v>
       </c>
       <c r="B14" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D14" s="6">
-        <v>230</v>
+        <v>151</v>
       </c>
       <c r="E14" s="6">
-        <v>309</v>
+        <v>229</v>
       </c>
       <c r="F14" s="7">
-        <v>681</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G14" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H14" s="8">
-        <v>6.9375</v>
+        <v>4.675</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>11</v>
@@ -1514,22 +1510,22 @@
         <v>4</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D15" s="6">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E15" s="6">
         <v>310</v>
       </c>
       <c r="F15" s="7">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="G15" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H15" s="8">
-        <v>6.9875</v>
+        <v>6.9375</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>11</v>
@@ -1543,22 +1539,22 @@
         <v>4</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D16" s="6">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E16" s="6">
         <v>309</v>
       </c>
       <c r="F16" s="7">
-        <v>685</v>
+        <v>681</v>
       </c>
       <c r="G16" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H16" s="8">
-        <v>6.9875</v>
+        <v>6.9375</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>11</v>
@@ -1569,25 +1565,25 @@
         <v>9</v>
       </c>
       <c r="B17" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D17" s="6">
-        <v>70</v>
+        <v>231</v>
       </c>
       <c r="E17" s="6">
-        <v>190</v>
+        <v>310</v>
       </c>
       <c r="F17" s="7">
-        <v>404</v>
+        <v>685</v>
       </c>
       <c r="G17" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H17" s="8">
-        <v>3.475</v>
+        <v>6.9875</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>11</v>
@@ -1598,25 +1594,25 @@
         <v>9</v>
       </c>
       <c r="B18" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D18" s="6">
-        <v>71</v>
+        <v>231</v>
       </c>
       <c r="E18" s="6">
-        <v>190</v>
+        <v>309</v>
       </c>
       <c r="F18" s="7">
-        <v>405</v>
+        <v>685</v>
       </c>
       <c r="G18" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H18" s="8">
-        <v>3.4875</v>
+        <v>6.9875</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>11</v>
@@ -1627,25 +1623,25 @@
         <v>9</v>
       </c>
       <c r="B19" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D19" s="6">
-        <v>150</v>
+        <v>-10</v>
       </c>
       <c r="E19" s="6">
-        <v>270</v>
+        <v>110</v>
       </c>
       <c r="F19" s="7">
-        <v>500.0000305176</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G19" s="7">
-        <v>817.9999389648</v>
+        <v>519.9999389648</v>
       </c>
       <c r="H19" s="8">
-        <v>4.675</v>
+        <v>3.425</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>11</v>
@@ -1656,25 +1652,25 @@
         <v>9</v>
       </c>
       <c r="B20" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D20" s="6">
-        <v>151</v>
+        <v>70</v>
       </c>
       <c r="E20" s="6">
-        <v>270</v>
+        <v>190</v>
       </c>
       <c r="F20" s="7">
-        <v>500.0000305176</v>
+        <v>404</v>
       </c>
       <c r="G20" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H20" s="8">
-        <v>4.675</v>
+        <v>3.475</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>11</v>
@@ -1685,25 +1681,25 @@
         <v>9</v>
       </c>
       <c r="B21" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D21" s="6">
-        <v>230</v>
+        <v>71</v>
       </c>
       <c r="E21" s="6">
-        <v>350</v>
+        <v>190</v>
       </c>
       <c r="F21" s="7">
-        <v>681</v>
+        <v>405</v>
       </c>
       <c r="G21" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H21" s="8">
-        <v>6.9375</v>
+        <v>3.4875</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>11</v>
@@ -1714,25 +1710,25 @@
         <v>9</v>
       </c>
       <c r="B22" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D22" s="6">
-        <v>231</v>
+        <v>150</v>
       </c>
       <c r="E22" s="6">
-        <v>350</v>
+        <v>270</v>
       </c>
       <c r="F22" s="7">
-        <v>685</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G22" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H22" s="8">
-        <v>6.9875</v>
+        <v>4.675</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>11</v>
@@ -1740,57 +1736,57 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="6" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B23" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D23" s="6">
-        <v>80</v>
+        <v>151</v>
       </c>
       <c r="E23" s="6">
-        <v>120</v>
+        <v>270</v>
       </c>
       <c r="F23" s="7">
-        <v>400.0000305176</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G23" s="7">
-        <v>451.9999694824</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H23" s="8">
-        <v>3.425</v>
-      </c>
-      <c r="I23" s="8">
-        <v>8.525</v>
+        <v>4.675</v>
+      </c>
+      <c r="I23" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="6" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B24" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="D24" s="6">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="E24" s="6">
-        <v>200</v>
+        <v>350</v>
       </c>
       <c r="F24" s="7">
-        <v>509</v>
+        <v>681</v>
       </c>
       <c r="G24" s="7">
-        <v>573.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H24" s="8">
-        <v>4.7875</v>
+        <v>6.9375</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>11</v>
@@ -1798,28 +1794,28 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="6" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B25" s="6">
         <v>4</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D25" s="6">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="E25" s="6">
-        <v>280</v>
+        <v>350</v>
       </c>
       <c r="F25" s="7">
-        <v>646</v>
+        <v>685</v>
       </c>
       <c r="G25" s="7">
-        <v>749.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H25" s="8">
-        <v>6.5</v>
+        <v>6.9875</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>11</v>
@@ -1830,28 +1826,28 @@
         <v>18</v>
       </c>
       <c r="B26" s="6">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D26" s="6">
-        <v>320</v>
+        <v>80</v>
       </c>
       <c r="E26" s="6">
-        <v>360</v>
+        <v>120</v>
       </c>
       <c r="F26" s="7">
-        <v>680.0000610352</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G26" s="7">
-        <v>817.9999389648</v>
+        <v>451.9999694824</v>
       </c>
       <c r="H26" s="8">
-        <v>6.925</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>11</v>
+        <v>3.425</v>
+      </c>
+      <c r="I26" s="8">
+        <v>8.525</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1859,25 +1855,25 @@
         <v>18</v>
       </c>
       <c r="B27" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D27" s="6">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="E27" s="6">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="F27" s="7">
-        <v>400.0000305176</v>
+        <v>509</v>
       </c>
       <c r="G27" s="7">
-        <v>496.9999694824</v>
+        <v>573.9999389648</v>
       </c>
       <c r="H27" s="8">
-        <v>3.425</v>
+        <v>4.7875</v>
       </c>
       <c r="I27" s="8" t="s">
         <v>11</v>
@@ -1888,25 +1884,25 @@
         <v>18</v>
       </c>
       <c r="B28" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D28" s="6">
-        <v>70</v>
+        <v>240</v>
       </c>
       <c r="E28" s="6">
-        <v>149</v>
+        <v>280</v>
       </c>
       <c r="F28" s="7">
-        <v>400.0000305176</v>
+        <v>646</v>
       </c>
       <c r="G28" s="7">
-        <v>492.9999694824</v>
+        <v>749.9999389648</v>
       </c>
       <c r="H28" s="8">
-        <v>3.425</v>
+        <v>6.5</v>
       </c>
       <c r="I28" s="8" t="s">
         <v>11</v>
@@ -1917,25 +1913,25 @@
         <v>18</v>
       </c>
       <c r="B29" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D29" s="6">
-        <v>71</v>
+        <v>320</v>
       </c>
       <c r="E29" s="6">
-        <v>150</v>
+        <v>360</v>
       </c>
       <c r="F29" s="7">
-        <v>400.0000305176</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G29" s="7">
-        <v>496.9999694824</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H29" s="8">
-        <v>3.425</v>
+        <v>6.925</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>11</v>
@@ -1949,19 +1945,19 @@
         <v>2</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D30" s="6">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E30" s="6">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F30" s="7">
         <v>400.0000305176</v>
       </c>
       <c r="G30" s="7">
-        <v>492.9999694824</v>
+        <v>496.9999694824</v>
       </c>
       <c r="H30" s="8">
         <v>3.425</v>
@@ -1975,25 +1971,25 @@
         <v>18</v>
       </c>
       <c r="B31" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D31" s="6">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="E31" s="6">
-        <v>230</v>
+        <v>149</v>
       </c>
       <c r="F31" s="7">
-        <v>493</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G31" s="7">
-        <v>630.9999389648</v>
+        <v>492.9999694824</v>
       </c>
       <c r="H31" s="8">
-        <v>4.5875</v>
+        <v>3.425</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>11</v>
@@ -2004,25 +2000,25 @@
         <v>18</v>
       </c>
       <c r="B32" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D32" s="6">
+        <v>71</v>
+      </c>
+      <c r="E32" s="6">
         <v>150</v>
       </c>
-      <c r="E32" s="6">
-        <v>229</v>
-      </c>
       <c r="F32" s="7">
-        <v>493</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G32" s="7">
-        <v>626.9999389648</v>
+        <v>496.9999694824</v>
       </c>
       <c r="H32" s="8">
-        <v>4.5875</v>
+        <v>3.425</v>
       </c>
       <c r="I32" s="8" t="s">
         <v>11</v>
@@ -2033,25 +2029,25 @@
         <v>18</v>
       </c>
       <c r="B33" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D33" s="6">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="E33" s="6">
-        <v>230</v>
+        <v>149</v>
       </c>
       <c r="F33" s="7">
-        <v>494</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G33" s="7">
-        <v>630.9999389648</v>
+        <v>492.9999694824</v>
       </c>
       <c r="H33" s="8">
-        <v>4.6</v>
+        <v>3.425</v>
       </c>
       <c r="I33" s="8" t="s">
         <v>11</v>
@@ -2065,22 +2061,22 @@
         <v>3</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D34" s="6">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E34" s="6">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F34" s="7">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="G34" s="7">
-        <v>626.9999389648</v>
+        <v>630.9999389648</v>
       </c>
       <c r="H34" s="8">
-        <v>4.6</v>
+        <v>4.5875</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>11</v>
@@ -2091,25 +2087,25 @@
         <v>18</v>
       </c>
       <c r="B35" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D35" s="6">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="E35" s="6">
-        <v>310</v>
+        <v>229</v>
       </c>
       <c r="F35" s="7">
-        <v>627</v>
+        <v>493</v>
       </c>
       <c r="G35" s="7">
-        <v>817.9999389648</v>
+        <v>626.9999389648</v>
       </c>
       <c r="H35" s="8">
-        <v>6.2625</v>
+        <v>4.5875</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>11</v>
@@ -2120,25 +2116,25 @@
         <v>18</v>
       </c>
       <c r="B36" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D36" s="6">
+        <v>151</v>
+      </c>
+      <c r="E36" s="6">
         <v>230</v>
       </c>
-      <c r="E36" s="6">
-        <v>309</v>
-      </c>
       <c r="F36" s="7">
-        <v>627</v>
+        <v>494</v>
       </c>
       <c r="G36" s="7">
-        <v>817.9999389648</v>
+        <v>630.9999389648</v>
       </c>
       <c r="H36" s="8">
-        <v>6.2625</v>
+        <v>4.6</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>11</v>
@@ -2149,25 +2145,25 @@
         <v>18</v>
       </c>
       <c r="B37" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D37" s="6">
-        <v>231</v>
+        <v>151</v>
       </c>
       <c r="E37" s="6">
-        <v>310</v>
+        <v>229</v>
       </c>
       <c r="F37" s="7">
-        <v>628</v>
+        <v>494</v>
       </c>
       <c r="G37" s="7">
-        <v>817.9999389648</v>
+        <v>626.9999389648</v>
       </c>
       <c r="H37" s="8">
-        <v>6.275</v>
+        <v>4.6</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>11</v>
@@ -2181,22 +2177,22 @@
         <v>4</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D38" s="6">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E38" s="6">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F38" s="7">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="G38" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H38" s="8">
-        <v>6.275</v>
+        <v>6.2625</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>11</v>
@@ -2207,25 +2203,25 @@
         <v>18</v>
       </c>
       <c r="B39" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D39" s="6">
-        <v>310</v>
+        <v>230</v>
       </c>
       <c r="E39" s="6">
-        <v>390</v>
+        <v>309</v>
       </c>
       <c r="F39" s="7">
-        <v>680.0000610352</v>
+        <v>627</v>
       </c>
       <c r="G39" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H39" s="8">
-        <v>6.925</v>
+        <v>6.2625</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>11</v>
@@ -2236,25 +2232,25 @@
         <v>18</v>
       </c>
       <c r="B40" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D40" s="6">
+        <v>231</v>
+      </c>
+      <c r="E40" s="6">
         <v>310</v>
       </c>
-      <c r="E40" s="6">
-        <v>389</v>
-      </c>
       <c r="F40" s="7">
-        <v>680.0000610352</v>
+        <v>628</v>
       </c>
       <c r="G40" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H40" s="8">
-        <v>6.925</v>
+        <v>6.275</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>11</v>
@@ -2265,25 +2261,25 @@
         <v>18</v>
       </c>
       <c r="B41" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D41" s="6">
-        <v>311</v>
+        <v>231</v>
       </c>
       <c r="E41" s="6">
-        <v>390</v>
+        <v>309</v>
       </c>
       <c r="F41" s="7">
-        <v>680.0000610352</v>
+        <v>628</v>
       </c>
       <c r="G41" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H41" s="8">
-        <v>6.925</v>
+        <v>6.275</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>11</v>
@@ -2297,13 +2293,13 @@
         <v>5</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D42" s="6">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E42" s="6">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F42" s="7">
         <v>680.0000610352</v>
@@ -2323,25 +2319,25 @@
         <v>18</v>
       </c>
       <c r="B43" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D43" s="6">
-        <v>390</v>
+        <v>310</v>
       </c>
       <c r="E43" s="6">
-        <v>470</v>
+        <v>389</v>
       </c>
       <c r="F43" s="7">
-        <v>796</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G43" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H43" s="8">
-        <v>8.375</v>
+        <v>6.925</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>11</v>
@@ -2352,25 +2348,25 @@
         <v>18</v>
       </c>
       <c r="B44" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D44" s="6">
+        <v>311</v>
+      </c>
+      <c r="E44" s="6">
         <v>390</v>
       </c>
-      <c r="E44" s="6">
-        <v>469</v>
-      </c>
       <c r="F44" s="7">
-        <v>796</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G44" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H44" s="8">
-        <v>8.375</v>
+        <v>6.925</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>11</v>
@@ -2381,25 +2377,25 @@
         <v>18</v>
       </c>
       <c r="B45" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D45" s="6">
-        <v>391</v>
+        <v>311</v>
       </c>
       <c r="E45" s="6">
-        <v>470</v>
+        <v>389</v>
       </c>
       <c r="F45" s="7">
-        <v>800</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G45" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H45" s="8">
-        <v>8.425</v>
+        <v>6.925</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>11</v>
@@ -2413,22 +2409,22 @@
         <v>6</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D46" s="6">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E46" s="6">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F46" s="7">
-        <v>800</v>
+        <v>796</v>
       </c>
       <c r="G46" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H46" s="8">
-        <v>8.425</v>
+        <v>8.375</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>11</v>
@@ -2439,25 +2435,25 @@
         <v>18</v>
       </c>
       <c r="B47" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D47" s="6">
-        <v>70</v>
+        <v>390</v>
       </c>
       <c r="E47" s="6">
-        <v>190</v>
+        <v>469</v>
       </c>
       <c r="F47" s="7">
-        <v>400.0000305176</v>
+        <v>796</v>
       </c>
       <c r="G47" s="7">
-        <v>557.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H47" s="8">
-        <v>3.425</v>
+        <v>8.375</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>11</v>
@@ -2468,25 +2464,25 @@
         <v>18</v>
       </c>
       <c r="B48" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D48" s="6">
-        <v>71</v>
+        <v>391</v>
       </c>
       <c r="E48" s="6">
-        <v>190</v>
+        <v>470</v>
       </c>
       <c r="F48" s="7">
-        <v>400.0000305176</v>
+        <v>800</v>
       </c>
       <c r="G48" s="7">
-        <v>557.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H48" s="8">
-        <v>3.425</v>
+        <v>8.425</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>11</v>
@@ -2497,25 +2493,25 @@
         <v>18</v>
       </c>
       <c r="B49" s="6">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D49" s="6">
-        <v>150</v>
+        <v>391</v>
       </c>
       <c r="E49" s="6">
-        <v>270</v>
+        <v>469</v>
       </c>
       <c r="F49" s="7">
-        <v>493</v>
+        <v>800</v>
       </c>
       <c r="G49" s="7">
-        <v>721.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H49" s="8">
-        <v>4.5875</v>
+        <v>8.425</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>11</v>
@@ -2526,28 +2522,28 @@
         <v>18</v>
       </c>
       <c r="B50" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D50" s="6">
-        <v>151</v>
+        <v>-10</v>
       </c>
       <c r="E50" s="6">
-        <v>270</v>
+        <v>110</v>
       </c>
       <c r="F50" s="7">
-        <v>494</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G50" s="7">
-        <v>721.9999389648</v>
+        <v>438.9999694824</v>
       </c>
       <c r="H50" s="8">
-        <v>4.6</v>
-      </c>
-      <c r="I50" s="8" t="s">
-        <v>11</v>
+        <v>3.425</v>
+      </c>
+      <c r="I50" s="8">
+        <v>8.3625</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2555,25 +2551,25 @@
         <v>18</v>
       </c>
       <c r="B51" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D51" s="6">
-        <v>230</v>
+        <v>70</v>
       </c>
       <c r="E51" s="6">
-        <v>350</v>
+        <v>190</v>
       </c>
       <c r="F51" s="7">
-        <v>627</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G51" s="7">
-        <v>817.9999389648</v>
+        <v>557.9999389648</v>
       </c>
       <c r="H51" s="8">
-        <v>6.2625</v>
+        <v>3.425</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>11</v>
@@ -2584,25 +2580,25 @@
         <v>18</v>
       </c>
       <c r="B52" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D52" s="6">
-        <v>231</v>
+        <v>71</v>
       </c>
       <c r="E52" s="6">
-        <v>350</v>
+        <v>190</v>
       </c>
       <c r="F52" s="7">
-        <v>628</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G52" s="7">
-        <v>817.9999389648</v>
+        <v>557.9999389648</v>
       </c>
       <c r="H52" s="8">
-        <v>6.275</v>
+        <v>3.425</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>11</v>
@@ -2613,25 +2609,25 @@
         <v>18</v>
       </c>
       <c r="B53" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D53" s="6">
-        <v>310</v>
+        <v>150</v>
       </c>
       <c r="E53" s="6">
-        <v>430</v>
+        <v>270</v>
       </c>
       <c r="F53" s="7">
-        <v>680.0000610352</v>
+        <v>493</v>
       </c>
       <c r="G53" s="7">
-        <v>817.9999389648</v>
+        <v>721.9999389648</v>
       </c>
       <c r="H53" s="8">
-        <v>6.925</v>
+        <v>4.5875</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>11</v>
@@ -2642,25 +2638,25 @@
         <v>18</v>
       </c>
       <c r="B54" s="6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D54" s="6">
-        <v>311</v>
+        <v>151</v>
       </c>
       <c r="E54" s="6">
-        <v>430</v>
+        <v>270</v>
       </c>
       <c r="F54" s="7">
-        <v>680.0000610352</v>
+        <v>494</v>
       </c>
       <c r="G54" s="7">
-        <v>817.9999389648</v>
+        <v>721.9999389648</v>
       </c>
       <c r="H54" s="8">
-        <v>6.925</v>
+        <v>4.6</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>11</v>
@@ -2671,25 +2667,25 @@
         <v>18</v>
       </c>
       <c r="B55" s="6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>16</v>
       </c>
       <c r="D55" s="6">
-        <v>390</v>
+        <v>230</v>
       </c>
       <c r="E55" s="6">
-        <v>510</v>
+        <v>350</v>
       </c>
       <c r="F55" s="7">
-        <v>796</v>
+        <v>627</v>
       </c>
       <c r="G55" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H55" s="8">
-        <v>8.375</v>
+        <v>6.2625</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>11</v>
@@ -2700,27 +2696,143 @@
         <v>18</v>
       </c>
       <c r="B56" s="6">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C56" s="6" t="s">
         <v>17</v>
       </c>
       <c r="D56" s="6">
+        <v>231</v>
+      </c>
+      <c r="E56" s="6">
+        <v>350</v>
+      </c>
+      <c r="F56" s="7">
+        <v>628</v>
+      </c>
+      <c r="G56" s="7">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H56" s="8">
+        <v>6.275</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" s="9">
+        <v>5</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D57" s="9">
+        <v>310</v>
+      </c>
+      <c r="E57" s="9">
+        <v>430</v>
+      </c>
+      <c r="F57" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G57" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H57" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" s="9">
+        <v>5</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D58" s="9">
+        <v>311</v>
+      </c>
+      <c r="E58" s="9">
+        <v>430</v>
+      </c>
+      <c r="F58" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G58" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H58" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I58" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B59" s="9">
+        <v>6</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="9">
+        <v>390</v>
+      </c>
+      <c r="E59" s="9">
+        <v>510</v>
+      </c>
+      <c r="F59" s="10">
+        <v>796</v>
+      </c>
+      <c r="G59" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H59" s="11">
+        <v>8.375</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" s="9">
+        <v>6</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D60" s="9">
         <v>391</v>
       </c>
-      <c r="E56" s="6">
+      <c r="E60" s="9">
         <v>510</v>
       </c>
-      <c r="F56" s="7">
+      <c r="F60" s="10">
         <v>800</v>
       </c>
-      <c r="G56" s="7">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H56" s="8">
+      <c r="G60" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H60" s="11">
         <v>8.425</v>
       </c>
-      <c r="I56" s="8" t="s">
+      <c r="I60" s="11" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
右侧南瓜修正 	modified:   "notebook/\345\260\217\351\254\274\350\220\275\347\202\271/\345\260\217\351\254\274\350\220\275\347\202\271.ipynb" 	modified:   "notebook/\345\260\217\351\254\274\350\220\275\347\202\271/\350\220\275\347\202\271\347\273\223\350\256\272.xlsx"
</commit_message>
<xml_diff>
--- a/notebook/小鬼落点/落点结论.xlsx
+++ b/notebook/小鬼落点/落点结论.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="21225" windowHeight="12615"/>
+    <workbookView windowHeight="17775" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="原始" sheetId="1" r:id="rId1"/>
+    <sheet name="右侧南瓜" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="25">
   <si>
     <t>场地</t>
   </si>
@@ -85,6 +86,24 @@
   <si>
     <t>屋顶</t>
   </si>
+  <si>
+    <t xml:space="preserve"> 普通 (</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 普通*(</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 炮尾 (</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 炮尾*(</t>
+  </si>
+  <si>
+    <t>*炮尾 (</t>
+  </si>
+  <si>
+    <t>*炮尾*(</t>
+  </si>
 </sst>
 </file>
 
@@ -98,7 +117,7 @@
     <numFmt numFmtId="176" formatCode="0.0000000000_ "/>
     <numFmt numFmtId="177" formatCode="0.0000_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -109,6 +128,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -591,133 +617,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -734,9 +760,9 @@
     <xf numFmtId="177" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="177" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1126,32 +1152,1791 @@
       </c>
     </row>
     <row r="2" spans="1:9">
+      <c r="A2" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="9">
+        <v>2</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="9">
+        <v>80</v>
+      </c>
+      <c r="E2" s="9">
+        <v>120</v>
+      </c>
+      <c r="F2" s="10">
+        <v>426</v>
+      </c>
+      <c r="G2" s="10">
+        <v>553.9999389648</v>
+      </c>
+      <c r="H2" s="11">
+        <v>3.75</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="9">
+        <v>3</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="9">
+        <v>160</v>
+      </c>
+      <c r="E3" s="9">
+        <v>200</v>
+      </c>
+      <c r="F3" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G3" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H3" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="9">
+        <v>4</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="9">
+        <v>240</v>
+      </c>
+      <c r="E4" s="9">
+        <v>280</v>
+      </c>
+      <c r="F4" s="10">
+        <v>727</v>
+      </c>
+      <c r="G4" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H4" s="11">
+        <v>7.5125</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="9">
+        <v>-10</v>
+      </c>
+      <c r="E5" s="9">
+        <v>70</v>
+      </c>
+      <c r="F5" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G5" s="10">
+        <v>407.9999694824</v>
+      </c>
+      <c r="H5" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I5" s="11">
+        <v>7.975</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="9">
+        <v>1</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="9">
+        <v>-10</v>
+      </c>
+      <c r="E6" s="9">
+        <v>69</v>
+      </c>
+      <c r="F6" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G6" s="10">
+        <v>406.9999694824</v>
+      </c>
+      <c r="H6" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I6" s="11">
+        <v>7.9625</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="9">
+        <v>2</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="9">
+        <v>70</v>
+      </c>
+      <c r="E7" s="9">
+        <v>150</v>
+      </c>
+      <c r="F7" s="10">
+        <v>404</v>
+      </c>
+      <c r="G7" s="10">
+        <v>700.9999389648</v>
+      </c>
+      <c r="H7" s="11">
+        <v>3.475</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="9">
+        <v>2</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="9">
+        <v>70</v>
+      </c>
+      <c r="E8" s="9">
+        <v>149</v>
+      </c>
+      <c r="F8" s="10">
+        <v>404</v>
+      </c>
+      <c r="G8" s="10">
+        <v>696.9999389648</v>
+      </c>
+      <c r="H8" s="11">
+        <v>3.475</v>
+      </c>
+      <c r="I8" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="9">
+        <v>2</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="9">
+        <v>71</v>
+      </c>
+      <c r="E9" s="9">
+        <v>150</v>
+      </c>
+      <c r="F9" s="10">
+        <v>405</v>
+      </c>
+      <c r="G9" s="10">
+        <v>700.9999389648</v>
+      </c>
+      <c r="H9" s="11">
+        <v>3.4875</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9">
+        <v>2</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="9">
+        <v>71</v>
+      </c>
+      <c r="E10" s="9">
+        <v>149</v>
+      </c>
+      <c r="F10" s="10">
+        <v>405</v>
+      </c>
+      <c r="G10" s="10">
+        <v>696.9999389648</v>
+      </c>
+      <c r="H10" s="11">
+        <v>3.4875</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="9">
+        <v>3</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="9">
+        <v>150</v>
+      </c>
+      <c r="E11" s="9">
+        <v>230</v>
+      </c>
+      <c r="F11" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G11" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H11" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="9">
+        <v>3</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="9">
+        <v>150</v>
+      </c>
+      <c r="E12" s="9">
+        <v>229</v>
+      </c>
+      <c r="F12" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G12" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H12" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9">
+        <v>3</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="9">
+        <v>151</v>
+      </c>
+      <c r="E13" s="9">
+        <v>230</v>
+      </c>
+      <c r="F13" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G13" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H13" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="9">
+        <v>3</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="9">
+        <v>151</v>
+      </c>
+      <c r="E14" s="9">
+        <v>229</v>
+      </c>
+      <c r="F14" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G14" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H14" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="9">
+        <v>4</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="9">
+        <v>230</v>
+      </c>
+      <c r="E15" s="9">
+        <v>310</v>
+      </c>
+      <c r="F15" s="10">
+        <v>681</v>
+      </c>
+      <c r="G15" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H15" s="11">
+        <v>6.9375</v>
+      </c>
+      <c r="I15" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="9">
+        <v>4</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="9">
+        <v>230</v>
+      </c>
+      <c r="E16" s="9">
+        <v>309</v>
+      </c>
+      <c r="F16" s="10">
+        <v>681</v>
+      </c>
+      <c r="G16" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H16" s="11">
+        <v>6.9375</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="9">
+        <v>4</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="9">
+        <v>231</v>
+      </c>
+      <c r="E17" s="9">
+        <v>310</v>
+      </c>
+      <c r="F17" s="10">
+        <v>685</v>
+      </c>
+      <c r="G17" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H17" s="11">
+        <v>6.9875</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="9">
+        <v>4</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="9">
+        <v>231</v>
+      </c>
+      <c r="E18" s="9">
+        <v>309</v>
+      </c>
+      <c r="F18" s="10">
+        <v>685</v>
+      </c>
+      <c r="G18" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H18" s="11">
+        <v>6.9875</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="9">
+        <v>1</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="9">
+        <v>-10</v>
+      </c>
+      <c r="E19" s="9">
+        <v>110</v>
+      </c>
+      <c r="F19" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G19" s="10">
+        <v>519.9999389648</v>
+      </c>
+      <c r="H19" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I19" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="9">
+        <v>2</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="9">
+        <v>70</v>
+      </c>
+      <c r="E20" s="9">
+        <v>190</v>
+      </c>
+      <c r="F20" s="10">
+        <v>404</v>
+      </c>
+      <c r="G20" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H20" s="11">
+        <v>3.475</v>
+      </c>
+      <c r="I20" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="9">
+        <v>2</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="9">
+        <v>71</v>
+      </c>
+      <c r="E21" s="9">
+        <v>190</v>
+      </c>
+      <c r="F21" s="10">
+        <v>405</v>
+      </c>
+      <c r="G21" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H21" s="11">
+        <v>3.4875</v>
+      </c>
+      <c r="I21" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B22" s="9">
+        <v>3</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="9">
+        <v>150</v>
+      </c>
+      <c r="E22" s="9">
+        <v>270</v>
+      </c>
+      <c r="F22" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G22" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H22" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I22" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" s="9">
+        <v>3</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="9">
+        <v>151</v>
+      </c>
+      <c r="E23" s="9">
+        <v>270</v>
+      </c>
+      <c r="F23" s="10">
+        <v>500.0000305176</v>
+      </c>
+      <c r="G23" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H23" s="11">
+        <v>4.675</v>
+      </c>
+      <c r="I23" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="9">
+        <v>4</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="9">
+        <v>230</v>
+      </c>
+      <c r="E24" s="9">
+        <v>350</v>
+      </c>
+      <c r="F24" s="10">
+        <v>681</v>
+      </c>
+      <c r="G24" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H24" s="11">
+        <v>6.9375</v>
+      </c>
+      <c r="I24" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" s="9">
+        <v>4</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="9">
+        <v>231</v>
+      </c>
+      <c r="E25" s="9">
+        <v>350</v>
+      </c>
+      <c r="F25" s="10">
+        <v>685</v>
+      </c>
+      <c r="G25" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H25" s="11">
+        <v>6.9875</v>
+      </c>
+      <c r="I25" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="9">
+        <v>2</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="9">
+        <v>80</v>
+      </c>
+      <c r="E26" s="9">
+        <v>120</v>
+      </c>
+      <c r="F26" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G26" s="10">
+        <v>451.9999694824</v>
+      </c>
+      <c r="H26" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I26" s="11">
+        <v>8.525</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="9">
+        <v>3</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="9">
+        <v>160</v>
+      </c>
+      <c r="E27" s="9">
+        <v>200</v>
+      </c>
+      <c r="F27" s="10">
+        <v>509</v>
+      </c>
+      <c r="G27" s="10">
+        <v>573.9999389648</v>
+      </c>
+      <c r="H27" s="11">
+        <v>4.7875</v>
+      </c>
+      <c r="I27" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B28" s="9">
+        <v>4</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="9">
+        <v>240</v>
+      </c>
+      <c r="E28" s="9">
+        <v>280</v>
+      </c>
+      <c r="F28" s="10">
+        <v>646</v>
+      </c>
+      <c r="G28" s="10">
+        <v>749.9999389648</v>
+      </c>
+      <c r="H28" s="11">
+        <v>6.5</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B29" s="9">
+        <v>5</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" s="9">
+        <v>320</v>
+      </c>
+      <c r="E29" s="9">
+        <v>360</v>
+      </c>
+      <c r="F29" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G29" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H29" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="9">
+        <v>2</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="9">
+        <v>70</v>
+      </c>
+      <c r="E30" s="9">
+        <v>150</v>
+      </c>
+      <c r="F30" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G30" s="10">
+        <v>496.9999694824</v>
+      </c>
+      <c r="H30" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="9">
+        <v>2</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="9">
+        <v>70</v>
+      </c>
+      <c r="E31" s="9">
+        <v>149</v>
+      </c>
+      <c r="F31" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G31" s="10">
+        <v>492.9999694824</v>
+      </c>
+      <c r="H31" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B32" s="9">
+        <v>2</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="9">
+        <v>71</v>
+      </c>
+      <c r="E32" s="9">
+        <v>150</v>
+      </c>
+      <c r="F32" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G32" s="10">
+        <v>496.9999694824</v>
+      </c>
+      <c r="H32" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I32" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B33" s="9">
+        <v>2</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="9">
+        <v>71</v>
+      </c>
+      <c r="E33" s="9">
+        <v>149</v>
+      </c>
+      <c r="F33" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G33" s="10">
+        <v>492.9999694824</v>
+      </c>
+      <c r="H33" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I33" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="9">
+        <v>3</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="9">
+        <v>150</v>
+      </c>
+      <c r="E34" s="9">
+        <v>230</v>
+      </c>
+      <c r="F34" s="10">
+        <v>493</v>
+      </c>
+      <c r="G34" s="10">
+        <v>630.9999389648</v>
+      </c>
+      <c r="H34" s="11">
+        <v>4.5875</v>
+      </c>
+      <c r="I34" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B35" s="9">
+        <v>3</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="9">
+        <v>150</v>
+      </c>
+      <c r="E35" s="9">
+        <v>229</v>
+      </c>
+      <c r="F35" s="10">
+        <v>493</v>
+      </c>
+      <c r="G35" s="10">
+        <v>626.9999389648</v>
+      </c>
+      <c r="H35" s="11">
+        <v>4.5875</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="9">
+        <v>3</v>
+      </c>
+      <c r="C36" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="9">
+        <v>151</v>
+      </c>
+      <c r="E36" s="9">
+        <v>230</v>
+      </c>
+      <c r="F36" s="10">
+        <v>494</v>
+      </c>
+      <c r="G36" s="10">
+        <v>630.9999389648</v>
+      </c>
+      <c r="H36" s="11">
+        <v>4.6</v>
+      </c>
+      <c r="I36" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B37" s="9">
+        <v>3</v>
+      </c>
+      <c r="C37" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D37" s="9">
+        <v>151</v>
+      </c>
+      <c r="E37" s="9">
+        <v>229</v>
+      </c>
+      <c r="F37" s="10">
+        <v>494</v>
+      </c>
+      <c r="G37" s="10">
+        <v>626.9999389648</v>
+      </c>
+      <c r="H37" s="11">
+        <v>4.6</v>
+      </c>
+      <c r="I37" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38" s="9">
+        <v>4</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" s="9">
+        <v>230</v>
+      </c>
+      <c r="E38" s="9">
+        <v>310</v>
+      </c>
+      <c r="F38" s="10">
+        <v>627</v>
+      </c>
+      <c r="G38" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H38" s="11">
+        <v>6.2625</v>
+      </c>
+      <c r="I38" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B39" s="9">
+        <v>4</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="9">
+        <v>230</v>
+      </c>
+      <c r="E39" s="9">
+        <v>309</v>
+      </c>
+      <c r="F39" s="10">
+        <v>627</v>
+      </c>
+      <c r="G39" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H39" s="11">
+        <v>6.2625</v>
+      </c>
+      <c r="I39" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B40" s="9">
+        <v>4</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="9">
+        <v>231</v>
+      </c>
+      <c r="E40" s="9">
+        <v>310</v>
+      </c>
+      <c r="F40" s="10">
+        <v>628</v>
+      </c>
+      <c r="G40" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H40" s="11">
+        <v>6.275</v>
+      </c>
+      <c r="I40" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="9">
+        <v>4</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" s="9">
+        <v>231</v>
+      </c>
+      <c r="E41" s="9">
+        <v>309</v>
+      </c>
+      <c r="F41" s="10">
+        <v>628</v>
+      </c>
+      <c r="G41" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H41" s="11">
+        <v>6.275</v>
+      </c>
+      <c r="I41" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B42" s="9">
+        <v>5</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" s="9">
+        <v>310</v>
+      </c>
+      <c r="E42" s="9">
+        <v>390</v>
+      </c>
+      <c r="F42" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G42" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H42" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I42" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43" s="9">
+        <v>5</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" s="9">
+        <v>310</v>
+      </c>
+      <c r="E43" s="9">
+        <v>389</v>
+      </c>
+      <c r="F43" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G43" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H43" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B44" s="9">
+        <v>5</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="9">
+        <v>311</v>
+      </c>
+      <c r="E44" s="9">
+        <v>390</v>
+      </c>
+      <c r="F44" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G44" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H44" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45" s="9">
+        <v>5</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D45" s="9">
+        <v>311</v>
+      </c>
+      <c r="E45" s="9">
+        <v>389</v>
+      </c>
+      <c r="F45" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G45" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H45" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I45" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46" s="9">
+        <v>6</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="9">
+        <v>390</v>
+      </c>
+      <c r="E46" s="9">
+        <v>470</v>
+      </c>
+      <c r="F46" s="10">
+        <v>796</v>
+      </c>
+      <c r="G46" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H46" s="11">
+        <v>8.375</v>
+      </c>
+      <c r="I46" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B47" s="9">
+        <v>6</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D47" s="9">
+        <v>390</v>
+      </c>
+      <c r="E47" s="9">
+        <v>469</v>
+      </c>
+      <c r="F47" s="10">
+        <v>796</v>
+      </c>
+      <c r="G47" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H47" s="11">
+        <v>8.375</v>
+      </c>
+      <c r="I47" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B48" s="9">
+        <v>6</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="9">
+        <v>391</v>
+      </c>
+      <c r="E48" s="9">
+        <v>470</v>
+      </c>
+      <c r="F48" s="10">
+        <v>800</v>
+      </c>
+      <c r="G48" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H48" s="11">
+        <v>8.425</v>
+      </c>
+      <c r="I48" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B49" s="9">
+        <v>6</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D49" s="9">
+        <v>391</v>
+      </c>
+      <c r="E49" s="9">
+        <v>469</v>
+      </c>
+      <c r="F49" s="10">
+        <v>800</v>
+      </c>
+      <c r="G49" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H49" s="11">
+        <v>8.425</v>
+      </c>
+      <c r="I49" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" s="9">
+        <v>1</v>
+      </c>
+      <c r="C50" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D50" s="9">
+        <v>-10</v>
+      </c>
+      <c r="E50" s="9">
+        <v>110</v>
+      </c>
+      <c r="F50" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G50" s="10">
+        <v>438.9999694824</v>
+      </c>
+      <c r="H50" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I50" s="11">
+        <v>8.3625</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B51" s="9">
+        <v>2</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D51" s="9">
+        <v>70</v>
+      </c>
+      <c r="E51" s="9">
+        <v>190</v>
+      </c>
+      <c r="F51" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G51" s="10">
+        <v>557.9999389648</v>
+      </c>
+      <c r="H51" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B52" s="9">
+        <v>2</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D52" s="9">
+        <v>71</v>
+      </c>
+      <c r="E52" s="9">
+        <v>190</v>
+      </c>
+      <c r="F52" s="10">
+        <v>400.0000305176</v>
+      </c>
+      <c r="G52" s="10">
+        <v>557.9999389648</v>
+      </c>
+      <c r="H52" s="11">
+        <v>3.425</v>
+      </c>
+      <c r="I52" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B53" s="9">
+        <v>3</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D53" s="9">
+        <v>150</v>
+      </c>
+      <c r="E53" s="9">
+        <v>270</v>
+      </c>
+      <c r="F53" s="10">
+        <v>493</v>
+      </c>
+      <c r="G53" s="10">
+        <v>721.9999389648</v>
+      </c>
+      <c r="H53" s="11">
+        <v>4.5875</v>
+      </c>
+      <c r="I53" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B54" s="9">
+        <v>3</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="9">
+        <v>151</v>
+      </c>
+      <c r="E54" s="9">
+        <v>270</v>
+      </c>
+      <c r="F54" s="10">
+        <v>494</v>
+      </c>
+      <c r="G54" s="10">
+        <v>721.9999389648</v>
+      </c>
+      <c r="H54" s="11">
+        <v>4.6</v>
+      </c>
+      <c r="I54" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B55" s="9">
+        <v>4</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D55" s="9">
+        <v>230</v>
+      </c>
+      <c r="E55" s="9">
+        <v>350</v>
+      </c>
+      <c r="F55" s="10">
+        <v>627</v>
+      </c>
+      <c r="G55" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H55" s="11">
+        <v>6.2625</v>
+      </c>
+      <c r="I55" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B56" s="9">
+        <v>4</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D56" s="9">
+        <v>231</v>
+      </c>
+      <c r="E56" s="9">
+        <v>350</v>
+      </c>
+      <c r="F56" s="10">
+        <v>628</v>
+      </c>
+      <c r="G56" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H56" s="11">
+        <v>6.275</v>
+      </c>
+      <c r="I56" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B57" s="9">
+        <v>5</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D57" s="9">
+        <v>310</v>
+      </c>
+      <c r="E57" s="9">
+        <v>430</v>
+      </c>
+      <c r="F57" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G57" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H57" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B58" s="9">
+        <v>5</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D58" s="9">
+        <v>311</v>
+      </c>
+      <c r="E58" s="9">
+        <v>430</v>
+      </c>
+      <c r="F58" s="10">
+        <v>680.0000610352</v>
+      </c>
+      <c r="G58" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H58" s="11">
+        <v>6.925</v>
+      </c>
+      <c r="I58" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B59" s="9">
+        <v>6</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D59" s="9">
+        <v>390</v>
+      </c>
+      <c r="E59" s="9">
+        <v>510</v>
+      </c>
+      <c r="F59" s="10">
+        <v>796</v>
+      </c>
+      <c r="G59" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H59" s="11">
+        <v>8.375</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B60" s="9">
+        <v>6</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D60" s="9">
+        <v>391</v>
+      </c>
+      <c r="E60" s="9">
+        <v>510</v>
+      </c>
+      <c r="F60" s="10">
+        <v>800</v>
+      </c>
+      <c r="G60" s="10">
+        <v>817.9999389648</v>
+      </c>
+      <c r="H60" s="11">
+        <v>8.425</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1:I53"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <cols>
+    <col min="1" max="2" width="5.375" customWidth="1"/>
+    <col min="3" max="3" width="7.125" customWidth="1"/>
+    <col min="4" max="5" width="17.75" customWidth="1"/>
+    <col min="6" max="7" width="20.25" style="1" customWidth="1"/>
+    <col min="8" max="9" width="11.5" style="2" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D2" s="6">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="E2" s="6">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="F2" s="7">
-        <v>426</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G2" s="7">
-        <v>553.9999389648</v>
+        <v>407.9999694824</v>
       </c>
       <c r="H2" s="8">
-        <v>3.75</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>11</v>
+        <v>3.425</v>
+      </c>
+      <c r="I2" s="8">
+        <v>7.975</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1159,28 +2944,28 @@
         <v>9</v>
       </c>
       <c r="B3" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D3" s="6">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="E3" s="6">
-        <v>200</v>
+        <v>69</v>
       </c>
       <c r="F3" s="7">
-        <v>500.0000305176</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G3" s="7">
-        <v>817.9999389648</v>
+        <v>406.9999694824</v>
       </c>
       <c r="H3" s="8">
-        <v>4.675</v>
-      </c>
-      <c r="I3" s="8" t="s">
-        <v>11</v>
+        <v>3.425</v>
+      </c>
+      <c r="I3" s="8">
+        <v>7.9625</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1188,25 +2973,25 @@
         <v>9</v>
       </c>
       <c r="B4" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D4" s="6">
-        <v>240</v>
+        <v>80</v>
       </c>
       <c r="E4" s="6">
-        <v>280</v>
+        <v>150</v>
       </c>
       <c r="F4" s="7">
-        <v>727</v>
+        <v>426</v>
       </c>
       <c r="G4" s="7">
-        <v>817.9999389648</v>
+        <v>700.9999389648</v>
       </c>
       <c r="H4" s="8">
-        <v>7.5125</v>
+        <v>3.75</v>
       </c>
       <c r="I4" s="8" t="s">
         <v>11</v>
@@ -1217,28 +3002,28 @@
         <v>9</v>
       </c>
       <c r="B5" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D5" s="6">
-        <v>-10</v>
+        <v>80</v>
       </c>
       <c r="E5" s="6">
-        <v>70</v>
+        <v>149</v>
       </c>
       <c r="F5" s="7">
-        <v>400.0000305176</v>
+        <v>426</v>
       </c>
       <c r="G5" s="7">
-        <v>407.9999694824</v>
+        <v>696.9999389648</v>
       </c>
       <c r="H5" s="8">
-        <v>3.425</v>
-      </c>
-      <c r="I5" s="8">
-        <v>7.975</v>
+        <v>3.75</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1246,28 +3031,28 @@
         <v>9</v>
       </c>
       <c r="B6" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D6" s="6">
-        <v>-10</v>
+        <v>160</v>
       </c>
       <c r="E6" s="6">
-        <v>69</v>
+        <v>230</v>
       </c>
       <c r="F6" s="7">
-        <v>400.0000305176</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G6" s="7">
-        <v>406.9999694824</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H6" s="8">
-        <v>3.425</v>
-      </c>
-      <c r="I6" s="8">
-        <v>7.9625</v>
+        <v>4.675</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1275,25 +3060,25 @@
         <v>9</v>
       </c>
       <c r="B7" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D7" s="6">
-        <v>70</v>
+        <v>160</v>
       </c>
       <c r="E7" s="6">
-        <v>150</v>
+        <v>229</v>
       </c>
       <c r="F7" s="7">
-        <v>404</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G7" s="7">
-        <v>700.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H7" s="8">
-        <v>3.475</v>
+        <v>4.675</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>11</v>
@@ -1304,25 +3089,25 @@
         <v>9</v>
       </c>
       <c r="B8" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D8" s="6">
-        <v>70</v>
+        <v>240</v>
       </c>
       <c r="E8" s="6">
-        <v>149</v>
+        <v>310</v>
       </c>
       <c r="F8" s="7">
-        <v>404</v>
+        <v>727</v>
       </c>
       <c r="G8" s="7">
-        <v>696.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H8" s="8">
-        <v>3.475</v>
+        <v>7.5125</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>11</v>
@@ -1333,25 +3118,25 @@
         <v>9</v>
       </c>
       <c r="B9" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D9" s="6">
-        <v>71</v>
+        <v>240</v>
       </c>
       <c r="E9" s="6">
-        <v>150</v>
+        <v>309</v>
       </c>
       <c r="F9" s="7">
-        <v>405</v>
+        <v>727</v>
       </c>
       <c r="G9" s="7">
-        <v>700.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H9" s="8">
-        <v>3.4875</v>
+        <v>7.5125</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>11</v>
@@ -1362,25 +3147,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D10" s="6">
-        <v>71</v>
+        <v>-10</v>
       </c>
       <c r="E10" s="6">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F10" s="7">
-        <v>405</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G10" s="7">
-        <v>696.9999389648</v>
+        <v>700.9999389648</v>
       </c>
       <c r="H10" s="8">
-        <v>3.4875</v>
+        <v>3.425</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>11</v>
@@ -1391,25 +3176,25 @@
         <v>9</v>
       </c>
       <c r="B11" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D11" s="6">
-        <v>150</v>
+        <v>-10</v>
       </c>
       <c r="E11" s="6">
-        <v>230</v>
+        <v>149</v>
       </c>
       <c r="F11" s="7">
-        <v>500.0000305176</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G11" s="7">
-        <v>817.9999389648</v>
+        <v>696.9999389648</v>
       </c>
       <c r="H11" s="8">
-        <v>4.675</v>
+        <v>3.425</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>11</v>
@@ -1420,25 +3205,25 @@
         <v>9</v>
       </c>
       <c r="B12" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D12" s="6">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="E12" s="6">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F12" s="7">
-        <v>500.0000305176</v>
+        <v>404</v>
       </c>
       <c r="G12" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H12" s="8">
-        <v>4.675</v>
+        <v>3.475</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>11</v>
@@ -1449,25 +3234,25 @@
         <v>9</v>
       </c>
       <c r="B13" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D13" s="6">
-        <v>151</v>
+        <v>70</v>
       </c>
       <c r="E13" s="6">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F13" s="7">
-        <v>500.0000305176</v>
+        <v>404</v>
       </c>
       <c r="G13" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H13" s="8">
-        <v>4.675</v>
+        <v>3.475</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>11</v>
@@ -1478,25 +3263,25 @@
         <v>9</v>
       </c>
       <c r="B14" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D14" s="6">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="E14" s="6">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F14" s="7">
-        <v>500.0000305176</v>
+        <v>405</v>
       </c>
       <c r="G14" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H14" s="8">
-        <v>4.675</v>
+        <v>3.4875</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>11</v>
@@ -1507,25 +3292,25 @@
         <v>9</v>
       </c>
       <c r="B15" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="D15" s="6">
-        <v>230</v>
+        <v>71</v>
       </c>
       <c r="E15" s="6">
-        <v>310</v>
+        <v>229</v>
       </c>
       <c r="F15" s="7">
-        <v>681</v>
+        <v>405</v>
       </c>
       <c r="G15" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H15" s="8">
-        <v>6.9375</v>
+        <v>3.4875</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>11</v>
@@ -1536,25 +3321,25 @@
         <v>9</v>
       </c>
       <c r="B16" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D16" s="6">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="E16" s="6">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F16" s="7">
-        <v>681</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G16" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H16" s="8">
-        <v>6.9375</v>
+        <v>4.675</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>11</v>
@@ -1565,25 +3350,25 @@
         <v>9</v>
       </c>
       <c r="B17" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D17" s="6">
-        <v>231</v>
+        <v>150</v>
       </c>
       <c r="E17" s="6">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F17" s="7">
-        <v>685</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G17" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H17" s="8">
-        <v>6.9875</v>
+        <v>4.675</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>11</v>
@@ -1594,25 +3379,25 @@
         <v>9</v>
       </c>
       <c r="B18" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D18" s="6">
-        <v>231</v>
+        <v>151</v>
       </c>
       <c r="E18" s="6">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F18" s="7">
-        <v>685</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G18" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H18" s="8">
-        <v>6.9875</v>
+        <v>4.675</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>11</v>
@@ -1623,25 +3408,25 @@
         <v>9</v>
       </c>
       <c r="B19" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D19" s="6">
-        <v>-10</v>
+        <v>151</v>
       </c>
       <c r="E19" s="6">
-        <v>110</v>
+        <v>309</v>
       </c>
       <c r="F19" s="7">
-        <v>400.0000305176</v>
+        <v>500.0000305176</v>
       </c>
       <c r="G19" s="7">
-        <v>519.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H19" s="8">
-        <v>3.425</v>
+        <v>4.675</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>11</v>
@@ -1652,25 +3437,25 @@
         <v>9</v>
       </c>
       <c r="B20" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D20" s="6">
-        <v>70</v>
+        <v>230</v>
       </c>
       <c r="E20" s="6">
-        <v>190</v>
+        <v>390</v>
       </c>
       <c r="F20" s="7">
-        <v>404</v>
+        <v>681</v>
       </c>
       <c r="G20" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H20" s="8">
-        <v>3.475</v>
+        <v>6.9375</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>11</v>
@@ -1681,25 +3466,25 @@
         <v>9</v>
       </c>
       <c r="B21" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D21" s="6">
-        <v>71</v>
+        <v>230</v>
       </c>
       <c r="E21" s="6">
-        <v>190</v>
+        <v>389</v>
       </c>
       <c r="F21" s="7">
-        <v>405</v>
+        <v>681</v>
       </c>
       <c r="G21" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H21" s="8">
-        <v>3.4875</v>
+        <v>6.9375</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>11</v>
@@ -1710,25 +3495,25 @@
         <v>9</v>
       </c>
       <c r="B22" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D22" s="6">
-        <v>150</v>
+        <v>231</v>
       </c>
       <c r="E22" s="6">
-        <v>270</v>
+        <v>390</v>
       </c>
       <c r="F22" s="7">
-        <v>500.0000305176</v>
+        <v>685</v>
       </c>
       <c r="G22" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H22" s="8">
-        <v>4.675</v>
+        <v>6.9875</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>11</v>
@@ -1739,25 +3524,25 @@
         <v>9</v>
       </c>
       <c r="B23" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D23" s="6">
-        <v>151</v>
+        <v>231</v>
       </c>
       <c r="E23" s="6">
-        <v>270</v>
+        <v>389</v>
       </c>
       <c r="F23" s="7">
-        <v>500.0000305176</v>
+        <v>685</v>
       </c>
       <c r="G23" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H23" s="8">
-        <v>4.675</v>
+        <v>6.9875</v>
       </c>
       <c r="I23" s="8" t="s">
         <v>11</v>
@@ -1765,28 +3550,28 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B24" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D24" s="6">
-        <v>230</v>
+        <v>80</v>
       </c>
       <c r="E24" s="6">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="F24" s="7">
-        <v>681</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G24" s="7">
-        <v>817.9999389648</v>
+        <v>496.9999694824</v>
       </c>
       <c r="H24" s="8">
-        <v>6.9375</v>
+        <v>3.425</v>
       </c>
       <c r="I24" s="8" t="s">
         <v>11</v>
@@ -1794,28 +3579,28 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="6" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B25" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D25" s="6">
-        <v>231</v>
+        <v>80</v>
       </c>
       <c r="E25" s="6">
-        <v>350</v>
+        <v>149</v>
       </c>
       <c r="F25" s="7">
-        <v>685</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G25" s="7">
-        <v>817.9999389648</v>
+        <v>492.9999694824</v>
       </c>
       <c r="H25" s="8">
-        <v>6.9875</v>
+        <v>3.425</v>
       </c>
       <c r="I25" s="8" t="s">
         <v>11</v>
@@ -1826,28 +3611,28 @@
         <v>18</v>
       </c>
       <c r="B26" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D26" s="6">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="E26" s="6">
-        <v>120</v>
+        <v>230</v>
       </c>
       <c r="F26" s="7">
-        <v>400.0000305176</v>
+        <v>509</v>
       </c>
       <c r="G26" s="7">
-        <v>451.9999694824</v>
+        <v>630.9999389648</v>
       </c>
       <c r="H26" s="8">
-        <v>3.425</v>
-      </c>
-      <c r="I26" s="8">
-        <v>8.525</v>
+        <v>4.7875</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1858,19 +3643,19 @@
         <v>3</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D27" s="6">
         <v>160</v>
       </c>
       <c r="E27" s="6">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="F27" s="7">
         <v>509</v>
       </c>
       <c r="G27" s="7">
-        <v>573.9999389648</v>
+        <v>626.9999389648</v>
       </c>
       <c r="H27" s="8">
         <v>4.7875</v>
@@ -1887,19 +3672,19 @@
         <v>4</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="D28" s="6">
         <v>240</v>
       </c>
       <c r="E28" s="6">
-        <v>280</v>
+        <v>310</v>
       </c>
       <c r="F28" s="7">
         <v>646</v>
       </c>
       <c r="G28" s="7">
-        <v>749.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H28" s="8">
         <v>6.5</v>
@@ -1913,25 +3698,25 @@
         <v>18</v>
       </c>
       <c r="B29" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D29" s="6">
-        <v>320</v>
+        <v>240</v>
       </c>
       <c r="E29" s="6">
-        <v>360</v>
+        <v>309</v>
       </c>
       <c r="F29" s="7">
-        <v>680.0000610352</v>
+        <v>646</v>
       </c>
       <c r="G29" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H29" s="8">
-        <v>6.925</v>
+        <v>6.5</v>
       </c>
       <c r="I29" s="8" t="s">
         <v>11</v>
@@ -1942,25 +3727,25 @@
         <v>18</v>
       </c>
       <c r="B30" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D30" s="6">
-        <v>70</v>
+        <v>320</v>
       </c>
       <c r="E30" s="6">
-        <v>150</v>
+        <v>390</v>
       </c>
       <c r="F30" s="7">
-        <v>400.0000305176</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G30" s="7">
-        <v>496.9999694824</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H30" s="8">
-        <v>3.425</v>
+        <v>6.925</v>
       </c>
       <c r="I30" s="8" t="s">
         <v>11</v>
@@ -1971,25 +3756,25 @@
         <v>18</v>
       </c>
       <c r="B31" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D31" s="6">
-        <v>70</v>
+        <v>320</v>
       </c>
       <c r="E31" s="6">
-        <v>149</v>
+        <v>389</v>
       </c>
       <c r="F31" s="7">
-        <v>400.0000305176</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G31" s="7">
-        <v>492.9999694824</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H31" s="8">
-        <v>3.425</v>
+        <v>6.925</v>
       </c>
       <c r="I31" s="8" t="s">
         <v>11</v>
@@ -2000,13 +3785,13 @@
         <v>18</v>
       </c>
       <c r="B32" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D32" s="6">
-        <v>71</v>
+        <v>-10</v>
       </c>
       <c r="E32" s="6">
         <v>150</v>
@@ -2029,13 +3814,13 @@
         <v>18</v>
       </c>
       <c r="B33" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D33" s="6">
-        <v>71</v>
+        <v>-10</v>
       </c>
       <c r="E33" s="6">
         <v>149</v>
@@ -2058,25 +3843,25 @@
         <v>18</v>
       </c>
       <c r="B34" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D34" s="6">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="E34" s="6">
         <v>230</v>
       </c>
       <c r="F34" s="7">
-        <v>493</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G34" s="7">
         <v>630.9999389648</v>
       </c>
       <c r="H34" s="8">
-        <v>4.5875</v>
+        <v>3.425</v>
       </c>
       <c r="I34" s="8" t="s">
         <v>11</v>
@@ -2087,25 +3872,25 @@
         <v>18</v>
       </c>
       <c r="B35" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D35" s="6">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="E35" s="6">
         <v>229</v>
       </c>
       <c r="F35" s="7">
-        <v>493</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G35" s="7">
         <v>626.9999389648</v>
       </c>
       <c r="H35" s="8">
-        <v>4.5875</v>
+        <v>3.425</v>
       </c>
       <c r="I35" s="8" t="s">
         <v>11</v>
@@ -2116,25 +3901,25 @@
         <v>18</v>
       </c>
       <c r="B36" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D36" s="6">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="E36" s="6">
         <v>230</v>
       </c>
       <c r="F36" s="7">
-        <v>494</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G36" s="7">
         <v>630.9999389648</v>
       </c>
       <c r="H36" s="8">
-        <v>4.6</v>
+        <v>3.425</v>
       </c>
       <c r="I36" s="8" t="s">
         <v>11</v>
@@ -2145,25 +3930,25 @@
         <v>18</v>
       </c>
       <c r="B37" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D37" s="6">
-        <v>151</v>
+        <v>71</v>
       </c>
       <c r="E37" s="6">
         <v>229</v>
       </c>
       <c r="F37" s="7">
-        <v>494</v>
+        <v>400.0000305176</v>
       </c>
       <c r="G37" s="7">
         <v>626.9999389648</v>
       </c>
       <c r="H37" s="8">
-        <v>4.6</v>
+        <v>3.425</v>
       </c>
       <c r="I37" s="8" t="s">
         <v>11</v>
@@ -2174,25 +3959,25 @@
         <v>18</v>
       </c>
       <c r="B38" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D38" s="6">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="E38" s="6">
         <v>310</v>
       </c>
       <c r="F38" s="7">
-        <v>627</v>
+        <v>493</v>
       </c>
       <c r="G38" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H38" s="8">
-        <v>6.2625</v>
+        <v>4.5875</v>
       </c>
       <c r="I38" s="8" t="s">
         <v>11</v>
@@ -2203,25 +3988,25 @@
         <v>18</v>
       </c>
       <c r="B39" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D39" s="6">
-        <v>230</v>
+        <v>150</v>
       </c>
       <c r="E39" s="6">
         <v>309</v>
       </c>
       <c r="F39" s="7">
-        <v>627</v>
+        <v>493</v>
       </c>
       <c r="G39" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H39" s="8">
-        <v>6.2625</v>
+        <v>4.5875</v>
       </c>
       <c r="I39" s="8" t="s">
         <v>11</v>
@@ -2232,25 +4017,25 @@
         <v>18</v>
       </c>
       <c r="B40" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D40" s="6">
-        <v>231</v>
+        <v>151</v>
       </c>
       <c r="E40" s="6">
         <v>310</v>
       </c>
       <c r="F40" s="7">
-        <v>628</v>
+        <v>494</v>
       </c>
       <c r="G40" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H40" s="8">
-        <v>6.275</v>
+        <v>4.6</v>
       </c>
       <c r="I40" s="8" t="s">
         <v>11</v>
@@ -2261,25 +4046,25 @@
         <v>18</v>
       </c>
       <c r="B41" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D41" s="6">
-        <v>231</v>
+        <v>151</v>
       </c>
       <c r="E41" s="6">
         <v>309</v>
       </c>
       <c r="F41" s="7">
-        <v>628</v>
+        <v>494</v>
       </c>
       <c r="G41" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H41" s="8">
-        <v>6.275</v>
+        <v>4.6</v>
       </c>
       <c r="I41" s="8" t="s">
         <v>11</v>
@@ -2290,25 +4075,25 @@
         <v>18</v>
       </c>
       <c r="B42" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D42" s="6">
-        <v>310</v>
+        <v>230</v>
       </c>
       <c r="E42" s="6">
         <v>390</v>
       </c>
       <c r="F42" s="7">
-        <v>680.0000610352</v>
+        <v>627</v>
       </c>
       <c r="G42" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H42" s="8">
-        <v>6.925</v>
+        <v>6.2625</v>
       </c>
       <c r="I42" s="8" t="s">
         <v>11</v>
@@ -2319,25 +4104,25 @@
         <v>18</v>
       </c>
       <c r="B43" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D43" s="6">
-        <v>310</v>
+        <v>230</v>
       </c>
       <c r="E43" s="6">
         <v>389</v>
       </c>
       <c r="F43" s="7">
-        <v>680.0000610352</v>
+        <v>627</v>
       </c>
       <c r="G43" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H43" s="8">
-        <v>6.925</v>
+        <v>6.2625</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>11</v>
@@ -2348,25 +4133,25 @@
         <v>18</v>
       </c>
       <c r="B44" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D44" s="6">
-        <v>311</v>
+        <v>231</v>
       </c>
       <c r="E44" s="6">
         <v>390</v>
       </c>
       <c r="F44" s="7">
-        <v>680.0000610352</v>
+        <v>628</v>
       </c>
       <c r="G44" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H44" s="8">
-        <v>6.925</v>
+        <v>6.275</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>11</v>
@@ -2377,25 +4162,25 @@
         <v>18</v>
       </c>
       <c r="B45" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D45" s="6">
-        <v>311</v>
+        <v>231</v>
       </c>
       <c r="E45" s="6">
         <v>389</v>
       </c>
       <c r="F45" s="7">
-        <v>680.0000610352</v>
+        <v>628</v>
       </c>
       <c r="G45" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H45" s="8">
-        <v>6.925</v>
+        <v>6.275</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>11</v>
@@ -2406,25 +4191,25 @@
         <v>18</v>
       </c>
       <c r="B46" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D46" s="6">
-        <v>390</v>
+        <v>310</v>
       </c>
       <c r="E46" s="6">
         <v>470</v>
       </c>
       <c r="F46" s="7">
-        <v>796</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G46" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H46" s="8">
-        <v>8.375</v>
+        <v>6.925</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>11</v>
@@ -2435,25 +4220,25 @@
         <v>18</v>
       </c>
       <c r="B47" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D47" s="6">
-        <v>390</v>
+        <v>310</v>
       </c>
       <c r="E47" s="6">
         <v>469</v>
       </c>
       <c r="F47" s="7">
-        <v>796</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G47" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H47" s="8">
-        <v>8.375</v>
+        <v>6.925</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>11</v>
@@ -2464,25 +4249,25 @@
         <v>18</v>
       </c>
       <c r="B48" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="D48" s="6">
-        <v>391</v>
+        <v>311</v>
       </c>
       <c r="E48" s="6">
         <v>470</v>
       </c>
       <c r="F48" s="7">
-        <v>800</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G48" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H48" s="8">
-        <v>8.425</v>
+        <v>6.925</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>11</v>
@@ -2493,25 +4278,25 @@
         <v>18</v>
       </c>
       <c r="B49" s="6">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="D49" s="6">
-        <v>391</v>
+        <v>311</v>
       </c>
       <c r="E49" s="6">
         <v>469</v>
       </c>
       <c r="F49" s="7">
-        <v>800</v>
+        <v>680.0000610352</v>
       </c>
       <c r="G49" s="7">
         <v>817.9999389648</v>
       </c>
       <c r="H49" s="8">
-        <v>8.425</v>
+        <v>6.925</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>11</v>
@@ -2522,28 +4307,28 @@
         <v>18</v>
       </c>
       <c r="B50" s="6">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D50" s="6">
-        <v>-10</v>
+        <v>390</v>
       </c>
       <c r="E50" s="6">
-        <v>110</v>
+        <v>550</v>
       </c>
       <c r="F50" s="7">
-        <v>400.0000305176</v>
+        <v>796</v>
       </c>
       <c r="G50" s="7">
-        <v>438.9999694824</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H50" s="8">
-        <v>3.425</v>
-      </c>
-      <c r="I50" s="8">
-        <v>8.3625</v>
+        <v>8.375</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2551,25 +4336,25 @@
         <v>18</v>
       </c>
       <c r="B51" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D51" s="6">
-        <v>70</v>
+        <v>390</v>
       </c>
       <c r="E51" s="6">
-        <v>190</v>
+        <v>549</v>
       </c>
       <c r="F51" s="7">
-        <v>400.0000305176</v>
+        <v>796</v>
       </c>
       <c r="G51" s="7">
-        <v>557.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H51" s="8">
-        <v>3.425</v>
+        <v>8.375</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>11</v>
@@ -2580,25 +4365,25 @@
         <v>18</v>
       </c>
       <c r="B52" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D52" s="6">
-        <v>71</v>
+        <v>391</v>
       </c>
       <c r="E52" s="6">
-        <v>190</v>
+        <v>550</v>
       </c>
       <c r="F52" s="7">
-        <v>400.0000305176</v>
+        <v>800</v>
       </c>
       <c r="G52" s="7">
-        <v>557.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H52" s="8">
-        <v>3.425</v>
+        <v>8.425</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>11</v>
@@ -2609,230 +4394,27 @@
         <v>18</v>
       </c>
       <c r="B53" s="6">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="D53" s="6">
-        <v>150</v>
+        <v>391</v>
       </c>
       <c r="E53" s="6">
-        <v>270</v>
+        <v>549</v>
       </c>
       <c r="F53" s="7">
-        <v>493</v>
+        <v>800</v>
       </c>
       <c r="G53" s="7">
-        <v>721.9999389648</v>
+        <v>817.9999389648</v>
       </c>
       <c r="H53" s="8">
-        <v>4.5875</v>
+        <v>8.425</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
-      <c r="A54" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B54" s="6">
-        <v>3</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D54" s="6">
-        <v>151</v>
-      </c>
-      <c r="E54" s="6">
-        <v>270</v>
-      </c>
-      <c r="F54" s="7">
-        <v>494</v>
-      </c>
-      <c r="G54" s="7">
-        <v>721.9999389648</v>
-      </c>
-      <c r="H54" s="8">
-        <v>4.6</v>
-      </c>
-      <c r="I54" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
-      <c r="A55" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B55" s="6">
-        <v>4</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D55" s="6">
-        <v>230</v>
-      </c>
-      <c r="E55" s="6">
-        <v>350</v>
-      </c>
-      <c r="F55" s="7">
-        <v>627</v>
-      </c>
-      <c r="G55" s="7">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H55" s="8">
-        <v>6.2625</v>
-      </c>
-      <c r="I55" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
-      <c r="A56" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B56" s="6">
-        <v>4</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D56" s="6">
-        <v>231</v>
-      </c>
-      <c r="E56" s="6">
-        <v>350</v>
-      </c>
-      <c r="F56" s="7">
-        <v>628</v>
-      </c>
-      <c r="G56" s="7">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H56" s="8">
-        <v>6.275</v>
-      </c>
-      <c r="I56" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
-      <c r="A57" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B57" s="9">
-        <v>5</v>
-      </c>
-      <c r="C57" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D57" s="9">
-        <v>310</v>
-      </c>
-      <c r="E57" s="9">
-        <v>430</v>
-      </c>
-      <c r="F57" s="10">
-        <v>680.0000610352</v>
-      </c>
-      <c r="G57" s="10">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H57" s="11">
-        <v>6.925</v>
-      </c>
-      <c r="I57" s="11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9">
-      <c r="A58" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B58" s="9">
-        <v>5</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D58" s="9">
-        <v>311</v>
-      </c>
-      <c r="E58" s="9">
-        <v>430</v>
-      </c>
-      <c r="F58" s="10">
-        <v>680.0000610352</v>
-      </c>
-      <c r="G58" s="10">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H58" s="11">
-        <v>6.925</v>
-      </c>
-      <c r="I58" s="11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
-      <c r="A59" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B59" s="9">
-        <v>6</v>
-      </c>
-      <c r="C59" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D59" s="9">
-        <v>390</v>
-      </c>
-      <c r="E59" s="9">
-        <v>510</v>
-      </c>
-      <c r="F59" s="10">
-        <v>796</v>
-      </c>
-      <c r="G59" s="10">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H59" s="11">
-        <v>8.375</v>
-      </c>
-      <c r="I59" s="11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9">
-      <c r="A60" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B60" s="9">
-        <v>6</v>
-      </c>
-      <c r="C60" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D60" s="9">
-        <v>391</v>
-      </c>
-      <c r="E60" s="9">
-        <v>510</v>
-      </c>
-      <c r="F60" s="10">
-        <v>800</v>
-      </c>
-      <c r="G60" s="10">
-        <v>817.9999389648</v>
-      </c>
-      <c r="H60" s="11">
-        <v>8.425</v>
-      </c>
-      <c r="I60" s="11" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>